<commit_message>
Fix date parsing and update mapbox token
Replace incorrect as.Date(..., "%m/%d/%y") parsing with explicit substring extraction and lubridate::make_date to build start_date/end_date, dropping temporary *_temp fields. Apply the same date fix in the server's clean_dat pipeline. Simplify mb_access_token call by removing install/overwrite arguments. Also include updated data assets (data/*.rds, codebook and www Excel) and add .DS_Store files.
</commit_message>
<xml_diff>
--- a/www/THRIVEair_codebook.xlsx
+++ b/www/THRIVEair_codebook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://drexel0-my.sharepoint.com/personal/lf649_drexel_edu/Documents/Research/South Philly R21/Report Back/Apps/THRIVEair_shiny/www/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lf649/git_repos/active/THRIVEair_shiny/www/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="117" documentId="8_{B2EB96DF-CBD3-5C4A-A150-B682CEB80B40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A0BDFA0-BBD1-1543-86D2-CA847FBDD13D}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04EABC3A-B136-BB42-BBF8-583DB2877DFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-35620" yWindow="-3100" windowWidth="34100" windowHeight="21020" xr2:uid="{FFB54211-1352-274A-AD01-EB240E61CC82}"/>
+    <workbookView xWindow="580" yWindow="500" windowWidth="34100" windowHeight="19680" xr2:uid="{FFB54211-1352-274A-AD01-EB240E61CC82}"/>
   </bookViews>
   <sheets>
     <sheet name="Codebook" sheetId="1" r:id="rId1"/>
@@ -53,9 +53,6 @@
     <t>Ethylbenzene</t>
   </si>
   <si>
-    <t>etbenz</t>
-  </si>
-  <si>
     <t>xylenes</t>
   </si>
   <si>
@@ -65,36 +62,15 @@
     <t>btex</t>
   </si>
   <si>
-    <t>mpxylene</t>
-  </si>
-  <si>
     <t>o-Xylene</t>
   </si>
   <si>
-    <t>oxylene</t>
-  </si>
-  <si>
     <t>1,2-dichlorobenzene</t>
   </si>
   <si>
-    <t>benz12chloro</t>
-  </si>
-  <si>
-    <t>benz1ethyl2methyl</t>
-  </si>
-  <si>
-    <t>benz1ethyl3methyl</t>
-  </si>
-  <si>
-    <t>benz1ethyl4methyl</t>
-  </si>
-  <si>
     <t>Propylbenzene</t>
   </si>
   <si>
-    <t>propylbenzene</t>
-  </si>
-  <si>
     <t>Decane</t>
   </si>
   <si>
@@ -113,12 +89,6 @@
     <t>heptane</t>
   </si>
   <si>
-    <t>heptane3methyl</t>
-  </si>
-  <si>
-    <t>hexane2methyl</t>
-  </si>
-  <si>
     <t>Mesitylene</t>
   </si>
   <si>
@@ -128,9 +98,6 @@
     <t>n-Hexane</t>
   </si>
   <si>
-    <t>hexane</t>
-  </si>
-  <si>
     <t>Nonane</t>
   </si>
   <si>
@@ -144,12 +111,6 @@
   </si>
   <si>
     <t>Tetrachloroethylene</t>
-  </si>
-  <si>
-    <t>tce</t>
-  </si>
-  <si>
-    <t>trichlorofluoromethane</t>
   </si>
   <si>
     <t>Undecane</t>
@@ -353,6 +314,45 @@
       </rPr>
       <t>Please note that values flagged LOD are detected, but at low concentrations. These values can be considered less accurate than values flagged REG.</t>
     </r>
+  </si>
+  <si>
+    <t>m_p_xylene_2</t>
+  </si>
+  <si>
+    <t>ethylbenzene</t>
+  </si>
+  <si>
+    <t>o_xylene</t>
+  </si>
+  <si>
+    <t>benzene_1_ethyl_2_methyl</t>
+  </si>
+  <si>
+    <t>benzene_1_ethyl_3_methyl</t>
+  </si>
+  <si>
+    <t>benzene_1_ethyl_4_methyl</t>
+  </si>
+  <si>
+    <t>benzene_propyl</t>
+  </si>
+  <si>
+    <t>n_hexane</t>
+  </si>
+  <si>
+    <t>hexane_2_methyl</t>
+  </si>
+  <si>
+    <t>heptane_3_methyl</t>
+  </si>
+  <si>
+    <t>benzene_1_2_dichloro</t>
+  </si>
+  <si>
+    <t>tetrachloroethylene</t>
+  </si>
+  <si>
+    <t>trichloromonofluoromethane</t>
   </si>
 </sst>
 </file>
@@ -507,7 +507,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
@@ -534,6 +534,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -561,13 +564,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -587,9 +583,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -627,7 +623,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -733,7 +729,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -875,7 +871,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -895,622 +891,621 @@
   <sheetData>
     <row r="1" spans="2:12" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:12" ht="26" x14ac:dyDescent="0.3">
-      <c r="B2" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="16"/>
+      <c r="B2" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="19"/>
       <c r="F2" s="10"/>
-      <c r="H2" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="I2" s="16"/>
+      <c r="H2" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="I2" s="19"/>
     </row>
     <row r="3" spans="2:12" ht="40" x14ac:dyDescent="0.25">
       <c r="B3" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="12" t="s">
         <v>42</v>
-      </c>
-      <c r="C3" s="27" t="s">
-        <v>40</v>
-      </c>
-      <c r="D3" s="27" t="s">
-        <v>41</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>55</v>
       </c>
       <c r="F3" s="7"/>
       <c r="H3" s="4" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B4" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="C4" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="23">
+        <v>47</v>
+      </c>
+      <c r="C4" t="s">
+        <v>88</v>
+      </c>
+      <c r="D4">
         <v>106.16</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="F4" s="1"/>
       <c r="H4" s="8" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B5" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C5" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="23">
+      <c r="D5">
         <v>78.11</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="F5" s="1"/>
       <c r="H5" s="8" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B6" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="23" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="23">
+      <c r="C6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D6">
         <v>106.17</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="F6" s="1"/>
       <c r="H6" s="8" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="2:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="23">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D7">
         <v>106.16</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="F7" s="1"/>
       <c r="H7" s="9" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="2:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="C8" t="s">
         <v>3</v>
       </c>
-      <c r="D8" s="23">
+      <c r="D8">
         <v>92.14</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="F8" s="1"/>
     </row>
     <row r="9" spans="2:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="23" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="23"/>
       <c r="E9" s="11" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="F9" s="1"/>
-      <c r="H9" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="I9" s="16"/>
+      <c r="H9" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="I9" s="19"/>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B10" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" s="23">
+        <v>48</v>
+      </c>
+      <c r="C10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10">
         <v>106.16</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="F10" s="1"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="18"/>
+      <c r="H10" s="20"/>
+      <c r="I10" s="21"/>
       <c r="L10" s="13"/>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B11" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="D11" s="23">
+        <v>49</v>
+      </c>
+      <c r="C11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11">
         <v>120.194</v>
       </c>
-      <c r="E11" s="24"/>
+      <c r="E11" s="14"/>
       <c r="F11" s="1"/>
-      <c r="H11" s="19" t="s">
-        <v>100</v>
-      </c>
-      <c r="I11" s="20"/>
+      <c r="H11" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="I11" s="23"/>
       <c r="L11" s="13"/>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B12" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="C12" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="D12" s="23">
+        <v>51</v>
+      </c>
+      <c r="C12" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12">
         <v>134.221</v>
       </c>
-      <c r="E12" s="24"/>
+      <c r="E12" s="14"/>
       <c r="F12" s="1"/>
-      <c r="H12" s="19"/>
-      <c r="I12" s="20"/>
+      <c r="H12" s="22"/>
+      <c r="I12" s="23"/>
       <c r="L12" s="13"/>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B13" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="C13" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="D13" s="23">
+        <v>53</v>
+      </c>
+      <c r="C13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D13">
         <v>120.19</v>
       </c>
-      <c r="E13" s="24"/>
+      <c r="E13" s="14"/>
       <c r="F13" s="1"/>
-      <c r="H13" s="19"/>
-      <c r="I13" s="20"/>
+      <c r="H13" s="22"/>
+      <c r="I13" s="23"/>
       <c r="L13" s="13"/>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B14" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="C14" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D14" s="23">
+        <v>54</v>
+      </c>
+      <c r="C14" t="s">
+        <v>92</v>
+      </c>
+      <c r="D14">
         <v>120.19</v>
       </c>
-      <c r="E14" s="24"/>
+      <c r="E14" s="14"/>
       <c r="F14" s="1"/>
-      <c r="H14" s="19"/>
-      <c r="I14" s="20"/>
+      <c r="H14" s="22"/>
+      <c r="I14" s="23"/>
       <c r="L14" s="13"/>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B15" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="C15" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="D15" s="23">
+        <v>55</v>
+      </c>
+      <c r="C15" t="s">
+        <v>93</v>
+      </c>
+      <c r="D15">
         <v>120.19</v>
       </c>
-      <c r="E15" s="24"/>
+      <c r="E15" s="14"/>
       <c r="F15" s="1"/>
-      <c r="H15" s="19"/>
-      <c r="I15" s="20"/>
+      <c r="H15" s="22"/>
+      <c r="I15" s="23"/>
       <c r="L15" s="13"/>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B16" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C16" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="23">
+        <v>17</v>
+      </c>
+      <c r="C16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16">
         <v>120.19</v>
       </c>
-      <c r="E16" s="24"/>
+      <c r="E16" s="14"/>
       <c r="F16" s="1"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="20"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="23"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B17" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C17" s="23" t="s">
-        <v>18</v>
-      </c>
-      <c r="D17" s="23">
+        <v>10</v>
+      </c>
+      <c r="C17" t="s">
+        <v>94</v>
+      </c>
+      <c r="D17">
         <v>120.19</v>
       </c>
-      <c r="E17" s="24"/>
+      <c r="E17" s="14"/>
       <c r="F17" s="1"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="20"/>
+      <c r="H17" s="22"/>
+      <c r="I17" s="23"/>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B18" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C18" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="D18" s="23">
+        <v>15</v>
+      </c>
+      <c r="C18" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18">
         <v>100.21</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="F18" s="1"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="20"/>
+      <c r="H18" s="22"/>
+      <c r="I18" s="23"/>
     </row>
     <row r="19" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B19" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C19" s="23" t="s">
-        <v>30</v>
-      </c>
-      <c r="D19" s="23">
+        <v>19</v>
+      </c>
+      <c r="C19" t="s">
+        <v>95</v>
+      </c>
+      <c r="D19">
         <v>86.18</v>
       </c>
-      <c r="E19" s="24"/>
+      <c r="E19" s="14"/>
       <c r="F19" s="1"/>
-      <c r="H19" s="21"/>
-      <c r="I19" s="22"/>
+      <c r="H19" s="24"/>
+      <c r="I19" s="25"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B20" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="C20" s="23" t="s">
-        <v>32</v>
-      </c>
-      <c r="D20" s="23">
+        <v>20</v>
+      </c>
+      <c r="C20" t="s">
+        <v>21</v>
+      </c>
+      <c r="D20">
         <v>128.25</v>
       </c>
-      <c r="E20" s="24"/>
+      <c r="E20" s="14"/>
       <c r="F20" s="1"/>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B21" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C21" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="D21" s="23">
+        <v>22</v>
+      </c>
+      <c r="C21" t="s">
+        <v>23</v>
+      </c>
+      <c r="D21">
         <v>114.23</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="F21" s="1"/>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B22" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C22" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="D22" s="23">
+        <v>11</v>
+      </c>
+      <c r="C22" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22">
         <v>149.29</v>
       </c>
-      <c r="E22" s="24"/>
+      <c r="E22" s="14"/>
       <c r="F22" s="1"/>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B23" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C23" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="D23" s="23">
+        <v>13</v>
+      </c>
+      <c r="C23" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23">
         <v>170.34</v>
       </c>
-      <c r="E23" s="24"/>
+      <c r="E23" s="14"/>
       <c r="F23" s="1"/>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B24" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="C24" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="D24" s="23">
+        <v>25</v>
+      </c>
+      <c r="C24" t="s">
+        <v>26</v>
+      </c>
+      <c r="D24">
         <v>156.31</v>
       </c>
-      <c r="E24" s="24"/>
+      <c r="E24" s="14"/>
       <c r="F24" s="1"/>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B25" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C25" s="23" t="s">
-        <v>70</v>
-      </c>
-      <c r="D25" s="23">
+        <v>56</v>
+      </c>
+      <c r="C25" t="s">
+        <v>57</v>
+      </c>
+      <c r="D25">
         <v>114.232</v>
       </c>
-      <c r="E25" s="24"/>
+      <c r="E25" s="14"/>
       <c r="F25" s="1"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B26" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="C26" s="23" t="s">
-        <v>72</v>
-      </c>
-      <c r="D26" s="23">
+        <v>58</v>
+      </c>
+      <c r="C26" t="s">
+        <v>59</v>
+      </c>
+      <c r="D26">
         <v>100.205</v>
       </c>
-      <c r="E26" s="24"/>
+      <c r="E26" s="14"/>
       <c r="F26" s="1"/>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B27" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="C27" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="D27" s="23">
+        <v>60</v>
+      </c>
+      <c r="C27" t="s">
+        <v>96</v>
+      </c>
+      <c r="D27">
         <v>100.2</v>
       </c>
-      <c r="E27" s="24"/>
+      <c r="E27" s="14"/>
       <c r="F27" s="1"/>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B28" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="C28" s="23" t="s">
-        <v>25</v>
-      </c>
-      <c r="D28" s="23">
+        <v>61</v>
+      </c>
+      <c r="C28" t="s">
+        <v>97</v>
+      </c>
+      <c r="D28">
         <v>114.23</v>
       </c>
-      <c r="E28" s="24"/>
+      <c r="E28" s="14"/>
       <c r="F28" s="1"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B29" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="C29" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="D29" s="23">
+        <v>62</v>
+      </c>
+      <c r="C29" t="s">
+        <v>63</v>
+      </c>
+      <c r="D29">
         <v>100.205</v>
       </c>
-      <c r="E29" s="24"/>
+      <c r="E29" s="14"/>
       <c r="F29" s="1"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B30" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="C30" s="23" t="s">
-        <v>78</v>
-      </c>
-      <c r="D30" s="23">
+        <v>64</v>
+      </c>
+      <c r="C30" t="s">
+        <v>65</v>
+      </c>
+      <c r="D30">
         <v>86.177999999999997</v>
       </c>
-      <c r="E30" s="24"/>
+      <c r="E30" s="14"/>
       <c r="F30" s="1"/>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B31" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="C31" s="23" t="s">
-        <v>80</v>
-      </c>
-      <c r="D31" s="23">
+        <v>66</v>
+      </c>
+      <c r="C31" t="s">
+        <v>67</v>
+      </c>
+      <c r="D31">
         <v>86.177999999999997</v>
       </c>
-      <c r="E31" s="24"/>
+      <c r="E31" s="14"/>
       <c r="F31" s="1"/>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B32" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="C32" s="23" t="s">
-        <v>82</v>
-      </c>
-      <c r="D32" s="23">
+        <v>68</v>
+      </c>
+      <c r="C32" t="s">
+        <v>69</v>
+      </c>
+      <c r="D32">
         <v>72.150999999999996</v>
       </c>
-      <c r="E32" s="24"/>
+      <c r="E32" s="14"/>
       <c r="F32" s="1"/>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B33" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="C33" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="D33" s="23">
+        <v>70</v>
+      </c>
+      <c r="C33" t="s">
+        <v>71</v>
+      </c>
+      <c r="D33">
         <v>98.188999999999993</v>
       </c>
-      <c r="E33" s="24"/>
+      <c r="E33" s="14"/>
       <c r="F33" s="1"/>
     </row>
     <row r="34" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B34" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C34" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="D34" s="23">
+        <v>72</v>
+      </c>
+      <c r="C34" t="s">
+        <v>73</v>
+      </c>
+      <c r="D34">
         <v>84.162000000000006</v>
       </c>
-      <c r="E34" s="24"/>
+      <c r="E34" s="14"/>
     </row>
     <row r="35" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B35" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="C35" s="23" t="s">
-        <v>88</v>
-      </c>
-      <c r="D35" s="23">
+        <v>74</v>
+      </c>
+      <c r="C35" t="s">
+        <v>75</v>
+      </c>
+      <c r="D35">
         <v>70.132900000000006</v>
       </c>
-      <c r="E35" s="24"/>
+      <c r="E35" s="14"/>
     </row>
     <row r="36" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B36" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="C36" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="D36" s="23">
+        <v>76</v>
+      </c>
+      <c r="C36" t="s">
+        <v>77</v>
+      </c>
+      <c r="D36">
         <v>68.12</v>
       </c>
-      <c r="E36" s="24"/>
+      <c r="E36" s="14"/>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B37" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="C37" s="23" t="s">
-        <v>92</v>
-      </c>
-      <c r="D37" s="23">
+        <v>78</v>
+      </c>
+      <c r="C37" t="s">
+        <v>79</v>
+      </c>
+      <c r="D37">
         <v>100.161</v>
       </c>
-      <c r="E37" s="24"/>
+      <c r="E37" s="14"/>
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B38" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="C38" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="D38" s="23">
+        <v>80</v>
+      </c>
+      <c r="C38" t="s">
+        <v>81</v>
+      </c>
+      <c r="D38">
         <v>100.16</v>
       </c>
-      <c r="E38" s="24"/>
+      <c r="E38" s="14"/>
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B39" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C39" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="D39" s="23">
+        <v>9</v>
+      </c>
+      <c r="C39" t="s">
+        <v>98</v>
+      </c>
+      <c r="D39">
         <v>147.01</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
     </row>
     <row r="40" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B40" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="C40" s="23" t="s">
-        <v>96</v>
-      </c>
-      <c r="D40" s="23">
+        <v>82</v>
+      </c>
+      <c r="C40" t="s">
+        <v>83</v>
+      </c>
+      <c r="D40">
         <v>153.81</v>
       </c>
-      <c r="E40" s="24"/>
+      <c r="E40" s="14"/>
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B41" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="C41" s="23" t="s">
-        <v>98</v>
-      </c>
-      <c r="D41" s="23">
+        <v>84</v>
+      </c>
+      <c r="C41" t="s">
+        <v>85</v>
+      </c>
+      <c r="D41">
         <v>119.37</v>
       </c>
-      <c r="E41" s="24"/>
+      <c r="E41" s="14"/>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B42" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C42" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="D42" s="23">
+        <v>24</v>
+      </c>
+      <c r="C42" t="s">
+        <v>99</v>
+      </c>
+      <c r="D42">
         <v>165.83</v>
       </c>
-      <c r="E42" s="24"/>
+      <c r="E42" s="14"/>
     </row>
     <row r="43" spans="2:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B43" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="C43" s="25" t="s">
-        <v>37</v>
-      </c>
-      <c r="D43" s="25">
+        <v>86</v>
+      </c>
+      <c r="C43" t="s">
+        <v>100</v>
+      </c>
+      <c r="D43" s="15">
         <v>137.37</v>
       </c>
-      <c r="E43" s="26"/>
+      <c r="E43" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>